<commit_message>
Updated incomplete database info
</commit_message>
<xml_diff>
--- a/Data/Terminator_Strength-250305.xlsx
+++ b/Data/Terminator_Strength-250305.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uob-my.sharepoint.com/personal/zw24976_bristol_ac_uk/Documents/Documents/BCL/PhagePol_Terminators/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="8_{2EA083DE-A26A-4505-B6D7-9B9BBECA4D55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{092D1982-CD55-4074-B8B7-DEDA37879B37}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="8_{2EA083DE-A26A-4505-B6D7-9B9BBECA4D55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B44A17AB-9D3B-4F69-877A-4DD7265E3956}"/>
   <bookViews>
-    <workbookView xWindow="-8910" yWindow="-21710" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{FBA8F37D-C457-492C-BCB7-AD86DC414F1B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FBA8F37D-C457-492C-BCB7-AD86DC414F1B}"/>
   </bookViews>
   <sheets>
-    <sheet name="OD600" sheetId="2" r:id="rId1"/>
-    <sheet name="GFP" sheetId="1" r:id="rId2"/>
-    <sheet name="RFP" sheetId="3" r:id="rId3"/>
+    <sheet name="PlateMap" sheetId="4" r:id="rId1"/>
+    <sheet name="OD600" sheetId="2" r:id="rId2"/>
+    <sheet name="GFP" sheetId="1" r:id="rId3"/>
+    <sheet name="RFP" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="0" hidden="1">'OD600'!$A$1:$CU$170</definedName>
+    <definedName name="ExternalData_1" localSheetId="1" hidden="1">'OD600'!$A$1:$CU$170</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14302" uniqueCount="9979">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14389" uniqueCount="10013">
   <si>
     <t/>
   </si>
@@ -29989,6 +29990,108 @@
   </si>
   <si>
     <t>3140</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>Blank</t>
+  </si>
+  <si>
+    <t>AF</t>
+  </si>
+  <si>
+    <t>0Cuma-TT7hyb1</t>
+  </si>
+  <si>
+    <t>0Cuma-noTer</t>
+  </si>
+  <si>
+    <t>0Cuma-RPU</t>
+  </si>
+  <si>
+    <t>1Cuma-TT7hyb1</t>
+  </si>
+  <si>
+    <t>1Cuma-noTer</t>
+  </si>
+  <si>
+    <t>1Cuma-RPU</t>
+  </si>
+  <si>
+    <t>2.5Cuma-TT7hyb1</t>
+  </si>
+  <si>
+    <t>2.5Cuma-noTer</t>
+  </si>
+  <si>
+    <t>2.5Cuma-RPU</t>
+  </si>
+  <si>
+    <t>5Cuma-TT7hyb1</t>
+  </si>
+  <si>
+    <t>5Cuma-noTer</t>
+  </si>
+  <si>
+    <t>5Cuma-RPU</t>
+  </si>
+  <si>
+    <t>10Cuma-TT7hyb1</t>
+  </si>
+  <si>
+    <t>10Cuma-noTer</t>
+  </si>
+  <si>
+    <t>10Cuma-RPU</t>
+  </si>
+  <si>
+    <t>25Cuma-TT7hyb1</t>
+  </si>
+  <si>
+    <t>25Cuma-noTer</t>
+  </si>
+  <si>
+    <t>25Cuma-RPU</t>
+  </si>
+  <si>
+    <t>50Cuma-TT7hyb1</t>
+  </si>
+  <si>
+    <t>50Cuma-noTer</t>
+  </si>
+  <si>
+    <t>50Cuma-RPU</t>
+  </si>
+  <si>
+    <t>100Cuma-TT7hyb1</t>
+  </si>
+  <si>
+    <t>100Cuma-noTer</t>
+  </si>
+  <si>
+    <t>100Cuma-RPU</t>
   </si>
 </sst>
 </file>
@@ -30364,10 +30467,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -30902,6 +31001,335 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD37B117-C6B0-4BA5-B1AA-D86A587A01FE}">
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="27" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
+      </c>
+      <c r="L1">
+        <v>11</v>
+      </c>
+      <c r="M1">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9979</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9989</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9989</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9989</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9990</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9990</v>
+      </c>
+      <c r="G2" t="s">
+        <v>9990</v>
+      </c>
+      <c r="H2" t="s">
+        <v>9991</v>
+      </c>
+      <c r="I2" t="s">
+        <v>9991</v>
+      </c>
+      <c r="J2" t="s">
+        <v>9991</v>
+      </c>
+      <c r="K2" t="s">
+        <v>9988</v>
+      </c>
+      <c r="L2" t="s">
+        <v>9988</v>
+      </c>
+      <c r="M2" t="s">
+        <v>9988</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9980</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9992</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9992</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9992</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9993</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9993</v>
+      </c>
+      <c r="G3" t="s">
+        <v>9993</v>
+      </c>
+      <c r="H3" t="s">
+        <v>9994</v>
+      </c>
+      <c r="I3" t="s">
+        <v>9994</v>
+      </c>
+      <c r="J3" t="s">
+        <v>9994</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9981</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9995</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9995</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9995</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9996</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9996</v>
+      </c>
+      <c r="G4" t="s">
+        <v>9996</v>
+      </c>
+      <c r="H4" t="s">
+        <v>9997</v>
+      </c>
+      <c r="I4" t="s">
+        <v>9997</v>
+      </c>
+      <c r="J4" t="s">
+        <v>9997</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9982</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9998</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9998</v>
+      </c>
+      <c r="D5" t="s">
+        <v>9998</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9999</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9999</v>
+      </c>
+      <c r="G5" t="s">
+        <v>9999</v>
+      </c>
+      <c r="H5" t="s">
+        <v>10000</v>
+      </c>
+      <c r="I5" t="s">
+        <v>10000</v>
+      </c>
+      <c r="J5" t="s">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9983</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10001</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10001</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10001</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10002</v>
+      </c>
+      <c r="F6" t="s">
+        <v>10002</v>
+      </c>
+      <c r="G6" t="s">
+        <v>10002</v>
+      </c>
+      <c r="H6" t="s">
+        <v>10003</v>
+      </c>
+      <c r="I6" t="s">
+        <v>10003</v>
+      </c>
+      <c r="J6" t="s">
+        <v>10003</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9984</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10004</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10004</v>
+      </c>
+      <c r="D7" t="s">
+        <v>10004</v>
+      </c>
+      <c r="E7" t="s">
+        <v>10005</v>
+      </c>
+      <c r="F7" t="s">
+        <v>10005</v>
+      </c>
+      <c r="G7" t="s">
+        <v>10005</v>
+      </c>
+      <c r="H7" t="s">
+        <v>10006</v>
+      </c>
+      <c r="I7" t="s">
+        <v>10006</v>
+      </c>
+      <c r="J7" t="s">
+        <v>10006</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>9985</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10007</v>
+      </c>
+      <c r="C8" t="s">
+        <v>10007</v>
+      </c>
+      <c r="D8" t="s">
+        <v>10007</v>
+      </c>
+      <c r="E8" t="s">
+        <v>10008</v>
+      </c>
+      <c r="F8" t="s">
+        <v>10008</v>
+      </c>
+      <c r="G8" t="s">
+        <v>10008</v>
+      </c>
+      <c r="H8" t="s">
+        <v>10009</v>
+      </c>
+      <c r="I8" t="s">
+        <v>10009</v>
+      </c>
+      <c r="J8" t="s">
+        <v>10009</v>
+      </c>
+      <c r="L8" t="s">
+        <v>9987</v>
+      </c>
+      <c r="M8" t="s">
+        <v>9987</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9986</v>
+      </c>
+      <c r="B9" t="s">
+        <v>10010</v>
+      </c>
+      <c r="C9" t="s">
+        <v>10010</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10010</v>
+      </c>
+      <c r="E9" t="s">
+        <v>10011</v>
+      </c>
+      <c r="F9" t="s">
+        <v>10011</v>
+      </c>
+      <c r="G9" t="s">
+        <v>10011</v>
+      </c>
+      <c r="H9" t="s">
+        <v>10012</v>
+      </c>
+      <c r="I9" t="s">
+        <v>10012</v>
+      </c>
+      <c r="J9" t="s">
+        <v>10012</v>
+      </c>
+      <c r="L9" t="s">
+        <v>9987</v>
+      </c>
+      <c r="M9" t="s">
+        <v>9987</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9E900EB-4AFE-41B6-80B5-BC84E7F3A37C}">
   <dimension ref="A1:CU50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -45873,7 +46301,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED18E39B-76DD-4E20-BA5F-2CE4D7CFD965}">
   <dimension ref="A1:CU50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -59189,7 +59617,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DC30E1B-1291-4F10-849D-024A25B32031}">
   <dimension ref="A1:CU50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>